<commit_message>
Archive cleanup: remove old daily outputs and retain fresh 2026-10-31 briefing
</commit_message>
<xml_diff>
--- a/output/PIB_UPSC_Daily_2026-10-31.xlsx
+++ b/output/PIB_UPSC_Daily_2026-10-31.xlsx
@@ -63,14 +63,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DCFCE7"/>
-        <bgColor rgb="00DCFCE7"/>
+        <fgColor rgb="00DBEAFE"/>
+        <bgColor rgb="00DBEAFE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DBEAFE"/>
-        <bgColor rgb="00DBEAFE"/>
+        <fgColor rgb="00DCFCE7"/>
+        <bgColor rgb="00DCFCE7"/>
       </patternFill>
     </fill>
     <fill>
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -558,12 +558,12 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Prime Minister's Office</t>
+          <t>President's Secretariat</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Prime Minister pays tribute to Sardar Vallabhbhai Patel on his birth anniversary</t>
+          <t>PRESIDENT OF INDIA PAYS FLORAL TRIBUTES TO SARDAR VALLABHBHAI PATEL ON HIS BIRTH ANNIVERSARY</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
@@ -578,7 +578,7 @@
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330739</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330757</t>
         </is>
       </c>
     </row>
@@ -588,32 +588,32 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>GS-3</t>
+          <t>GS-2</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Prime Minister's Office</t>
+          <t>Lok Sabha Secretariat</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>PM congratulates ISRO scientists and engineers on successful launch of GSLV-F18 carrying NVS-03</t>
+          <t>LOK SABHA SPEAKER HAILS GAYATRI PARIVAR’S CONTRIBUTIONS TO INDIA'S SPIRITUAL RENAISSANCE, SOCIAL TRANSFORMATION AND NATION-BUILDING</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>isro, gslv, nvs</t>
+          <t>lok sabha</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 3 topics: isro, gslv, nvs</t>
+          <t>Aligned with General Studies 2 topics: lok sabha</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330735</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330789</t>
         </is>
       </c>
     </row>
@@ -621,34 +621,34 @@
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>GS-3</t>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>GS-1</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Ministry of Home Affairs</t>
+          <t>Prime Minister's Office</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>‘Kendriya Grihmantri Dakshata Padak’ awarded to 490 personnel of various States/UTs/CAPFs/CPOs for the year 2026</t>
+          <t>Prime Minister pays tribute to Sardar Vallabhbhai Patel on his birth anniversary</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>dakshata padak, kendriya grihmantri dakshata padak, capfs, cpos</t>
+          <t>birth anniversary, sardar vallabhbhai patel</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 3 topics: dakshata padak, kendriya grihmantri dakshata padak, capfs</t>
+          <t>Aligned with General Studies 1 topics: birth anniversary, sardar vallabhbhai patel</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330728</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330739</t>
         </is>
       </c>
     </row>
@@ -658,32 +658,32 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>GS-2</t>
+          <t>GS-3</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Ministry of Rural Development</t>
+          <t>Prime Minister's Office</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Mizoram Gets Approval for New Road Works under PMGSY-IV to Strengthen Rural Connectivity</t>
+          <t>PM congratulates ISRO scientists and engineers on successful launch of GSLV-F18 carrying NVS-03</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>pmgsy, pmgsy-iv, rural connectivity</t>
+          <t>isro, gslv, nvs</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 2 topics: pmgsy, pmgsy-iv, rural connectivity</t>
+          <t>Aligned with General Studies 3 topics: isro, gslv, nvs</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330725</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330735</t>
         </is>
       </c>
     </row>
@@ -691,32 +691,243 @@
       <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>GS-1</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>AYUSH</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Ayush Promotes ‘Yoga for Unity’ on National Unity Day 2026</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>national unity day</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 1 topics: national unity day</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330770</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Agriculture &amp;
+Farmers Welfare</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>DARE–ICAR Intensifies Special Campaign 6.0, Promotes Cleanliness, Sustainable Waste Management and Better Office Spaces Across Institutes</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>agriculture</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 3 topics: agriculture</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330771</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>GS-1</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Health and Family Welfare</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Union Health Minister Shri J.P. Nadda administers Rashtriya Ekta Diwas pledge to commemorate the birth anniversary of Sardar Vallabhbhai Patel</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>birth anniversary, rashtriya ekta diwas, sardar vallabhbhai patel</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 1 topics: birth anniversary, rashtriya ekta diwas, sardar vallabhbhai patel</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330752</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Home Affairs</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>‘Kendriya Grihmantri Dakshata Padak’ awarded to 490 personnel of various States/UTs/CAPFs/CPOs for the year 2026</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>dakshata padak, kendriya grihmantri dakshata padak, capfs, cpos</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 3 topics: dakshata padak, kendriya grihmantri dakshata padak, capfs</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330728</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>GS-2</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Panchayati Raj</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Union Minister Shri Rajiv Ranjan Singh Urges Concerted Efforts to Build ‘Atmanirbhar Panchayats’ at National Workshop on People’s Plan Campaign, in New Delhi</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>panchayati raj</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 2 topics: panchayati raj</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330751</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>GS-2</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Rural Development</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Mizoram Gets Approval for New Road Works under PMGSY-IV to Strengthen Rural Connectivity</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>pmgsy, pmgsy-iv, rural connectivity</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 2 topics: pmgsy, pmgsy-iv, rural connectivity</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330725</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>GS-2</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>PIB Backgrounder</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>India’s Social Security Coverage</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>PIB Backgrounder, social security</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>PIB Backgrounder: Aligned with General Studies 2 topics: social security</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G12" s="5" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330727</t>
         </is>
@@ -729,6 +940,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -740,7 +957,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -799,17 +1016,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Prime Minister's Office</t>
+          <t>President's Secretariat</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Prime Minister pays tribute to Sardar Vallabhbhai Patel on his birth anniversary</t>
+          <t>PRESIDENT OF INDIA PAYS FLORAL TRIBUTES TO SARDAR VALLABHBHAI PATEL ON HIS BIRTH ANNIVERSARY</t>
         </is>
       </c>
       <c r="F2" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330739</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330757</t>
         </is>
       </c>
     </row>
@@ -824,22 +1041,22 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>GS-3</t>
+          <t>GS-2</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Prime Minister's Office</t>
+          <t>Lok Sabha Secretariat</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>PM congratulates ISRO scientists and engineers on successful launch of GSLV-F18 carrying NVS-03</t>
+          <t>LOK SABHA SPEAKER HAILS GAYATRI PARIVAR’S CONTRIBUTIONS TO INDIA'S SPIRITUAL RENAISSANCE, SOCIAL TRANSFORMATION AND NATION-BUILDING</t>
         </is>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330735</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330789</t>
         </is>
       </c>
     </row>
@@ -854,22 +1071,22 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>GS-3</t>
+          <t>GS-1</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Ministry of Home Affairs</t>
+          <t>Prime Minister's Office</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>‘Kendriya Grihmantri Dakshata Padak’ awarded to 490 personnel of various States/UTs/CAPFs/CPOs for the year 2026</t>
+          <t>Prime Minister pays tribute to Sardar Vallabhbhai Patel on his birth anniversary</t>
         </is>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330728</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330739</t>
         </is>
       </c>
     </row>
@@ -884,22 +1101,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>GS-2</t>
+          <t>GS-3</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Ministry of Rural Development</t>
+          <t>Prime Minister's Office</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Mizoram Gets Approval for New Road Works under PMGSY-IV to Strengthen Rural Connectivity</t>
+          <t>PM congratulates ISRO scientists and engineers on successful launch of GSLV-F18 carrying NVS-03</t>
         </is>
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330725</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330735</t>
         </is>
       </c>
     </row>
@@ -909,27 +1126,27 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Routine Fluff</t>
+          <t>Relevant (UPSC)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>General/Administrative</t>
+          <t>GS-1</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Ministry of Textiles</t>
+          <t>AYUSH</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Prime Minister visits CCIC Pavilion at Bharat Parv 2026 in Ekta Nagar, Gujarat</t>
+          <t>Ministry of Ayush Promotes ‘Yoga for Unity’ on National Unity Day 2026</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330737</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330770</t>
         </is>
       </c>
     </row>
@@ -944,20 +1161,201 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Ministry of Agriculture &amp;
+Farmers Welfare</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>DARE–ICAR Intensifies Special Campaign 6.0, Promotes Cleanliness, Sustainable Waste Management and Better Office Spaces Across Institutes</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330771</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>GS-1</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Ministry of Health and Family Welfare</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Union Health Minister Shri J.P. Nadda administers Rashtriya Ekta Diwas pledge to commemorate the birth anniversary of Sardar Vallabhbhai Patel</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330752</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Ministry of Home Affairs</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>‘Kendriya Grihmantri Dakshata Padak’ awarded to 490 personnel of various States/UTs/CAPFs/CPOs for the year 2026</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330728</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
           <t>GS-2</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Ministry of Panchayati Raj</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Union Minister Shri Rajiv Ranjan Singh Urges Concerted Efforts to Build ‘Atmanirbhar Panchayats’ at National Workshop on People’s Plan Campaign, in New Delhi</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330751</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>GS-2</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Ministry of Rural Development</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Mizoram Gets Approval for New Road Works under PMGSY-IV to Strengthen Rural Connectivity</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330725</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Ministry of Textiles</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Prime Minister visits CCIC Pavilion at Bharat Parv 2026 in Ekta Nagar, Gujarat</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330737</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>GS-2</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
         <is>
           <t>PIB Backgrounder</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>India’s Social Security Coverage</t>
         </is>
       </c>
-      <c r="F7" s="9" t="inlineStr">
+      <c r="F13" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330727</t>
         </is>
@@ -971,6 +1369,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto-archive: Daily PIB UPSC Brief 2026-11-01
</commit_message>
<xml_diff>
--- a/output/PIB_UPSC_Daily_2026-10-31.xlsx
+++ b/output/PIB_UPSC_Daily_2026-10-31.xlsx
@@ -63,14 +63,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DBEAFE"/>
-        <bgColor rgb="00DBEAFE"/>
+        <fgColor rgb="00DCFCE7"/>
+        <bgColor rgb="00DCFCE7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DCFCE7"/>
-        <bgColor rgb="00DCFCE7"/>
+        <fgColor rgb="00DBEAFE"/>
+        <bgColor rgb="00DBEAFE"/>
       </patternFill>
     </fill>
     <fill>
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -586,34 +586,34 @@
       <c r="A3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>GS-2</t>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>GS-1</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Lok Sabha Secretariat</t>
+          <t>Vice President's Secretariat</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>LOK SABHA SPEAKER HAILS GAYATRI PARIVAR’S CONTRIBUTIONS TO INDIA'S SPIRITUAL RENAISSANCE, SOCIAL TRANSFORMATION AND NATION-BUILDING</t>
+          <t>Vice-President Shri C. P. Radhakrishnan attends ‘Sardar Katha’ at Uprashtrapati Bhavan; pays tribute to Sardar Vallabhbhai Patel on Rashtriya Ekta Diwas</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>lok sabha</t>
+          <t>rashtriya ekta diwas, sardar vallabhbhai patel</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 2 topics: lok sabha</t>
+          <t>Aligned with General Studies 1 topics: rashtriya ekta diwas, sardar vallabhbhai patel</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330789</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330939</t>
         </is>
       </c>
     </row>
@@ -633,22 +633,22 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Prime Minister pays tribute to Sardar Vallabhbhai Patel on his birth anniversary</t>
+          <t>English rendering of PM’s speech at the Rashtriya Ekta Diwas programme in Kevadia, Gujarat</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>birth anniversary, sardar vallabhbhai patel</t>
+          <t>rashtriya ekta diwas</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 1 topics: birth anniversary, sardar vallabhbhai patel</t>
+          <t>Aligned with General Studies 1 topics: rashtriya ekta diwas</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330739</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2331035</t>
         </is>
       </c>
     </row>
@@ -656,9 +656,9 @@
       <c r="A5" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>GS-3</t>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>GS-1</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -668,22 +668,22 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>PM congratulates ISRO scientists and engineers on successful launch of GSLV-F18 carrying NVS-03</t>
+          <t>Prime Minister Shri Narendra Modi participates in Rashtriya Ekta Diwas Celebrations marking the 151st birth anniversary of Sardar Vallabhbhai Patel</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>isro, gslv, nvs</t>
+          <t>birth anniversary, rashtriya ekta diwas, sardar vallabhbhai patel</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 3 topics: isro, gslv, nvs</t>
+          <t>Aligned with General Studies 1 topics: birth anniversary, rashtriya ekta diwas, sardar vallabhbhai patel</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330735</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2331033</t>
         </is>
       </c>
     </row>
@@ -698,27 +698,27 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>AYUSH</t>
+          <t>Prime Minister's Office</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Ministry of Ayush Promotes ‘Yoga for Unity’ on National Unity Day 2026</t>
+          <t>Prime Minister pays tribute to Sardar Vallabhbhai Patel on his birth anniversary</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>national unity day</t>
+          <t>birth anniversary, sardar vallabhbhai patel</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 1 topics: national unity day</t>
+          <t>Aligned with General Studies 1 topics: birth anniversary, sardar vallabhbhai patel</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330770</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330739</t>
         </is>
       </c>
     </row>
@@ -726,35 +726,34 @@
       <c r="A7" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>GS-3</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Ministry of Agriculture &amp;
-Farmers Welfare</t>
+          <t>Prime Minister's Office</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>DARE–ICAR Intensifies Special Campaign 6.0, Promotes Cleanliness, Sustainable Waste Management and Better Office Spaces Across Institutes</t>
+          <t>PM congratulates ISRO scientists and engineers on successful launch of GSLV-F18 carrying NVS-03</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>agriculture</t>
+          <t>isro, gslv, nvs</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 3 topics: agriculture</t>
+          <t>Aligned with General Studies 3 topics: isro, gslv, nvs</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330771</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330735</t>
         </is>
       </c>
     </row>
@@ -762,34 +761,34 @@
       <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>GS-1</t>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>GS-2</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Ministry of Health and Family Welfare</t>
+          <t>Lok Sabha Secretariat</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Union Health Minister Shri J.P. Nadda administers Rashtriya Ekta Diwas pledge to commemorate the birth anniversary of Sardar Vallabhbhai Patel</t>
+          <t>LOK SABHA SPEAKER HAILS GAYATRI PARIVAR’S CONTRIBUTIONS TO INDIA'S SPIRITUAL RENAISSANCE, SOCIAL TRANSFORMATION AND NATION-BUILDING</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>birth anniversary, rashtriya ekta diwas, sardar vallabhbhai patel</t>
+          <t>lok sabha</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 1 topics: birth anniversary, rashtriya ekta diwas, sardar vallabhbhai patel</t>
+          <t>Aligned with General Studies 2 topics: lok sabha</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330752</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330789</t>
         </is>
       </c>
     </row>
@@ -797,34 +796,34 @@
       <c r="A9" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>GS-3</t>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>GS-1</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Ministry of Home Affairs</t>
+          <t>AYUSH</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>‘Kendriya Grihmantri Dakshata Padak’ awarded to 490 personnel of various States/UTs/CAPFs/CPOs for the year 2026</t>
+          <t>Ministry of Ayush Promotes ‘Yoga for Unity’ on National Unity Day 2026</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>dakshata padak, kendriya grihmantri dakshata padak, capfs, cpos</t>
+          <t>national unity day</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 3 topics: dakshata padak, kendriya grihmantri dakshata padak, capfs</t>
+          <t>Aligned with General Studies 1 topics: national unity day</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330728</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330770</t>
         </is>
       </c>
     </row>
@@ -834,32 +833,33 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>GS-2</t>
+          <t>GS-3</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Ministry of Panchayati Raj</t>
+          <t>Ministry of Agriculture &amp;
+Farmers Welfare</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Union Minister Shri Rajiv Ranjan Singh Urges Concerted Efforts to Build ‘Atmanirbhar Panchayats’ at National Workshop on People’s Plan Campaign, in New Delhi</t>
+          <t>DARE–ICAR Intensifies Special Campaign 6.0, Promotes Cleanliness, Sustainable Waste Management and Better Office Spaces Across Institutes</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>panchayati raj</t>
+          <t>agriculture</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 2 topics: panchayati raj</t>
+          <t>Aligned with General Studies 3 topics: agriculture</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330751</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330771</t>
         </is>
       </c>
     </row>
@@ -869,32 +869,32 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>GS-2</t>
+          <t>GS-3</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Ministry of Rural Development</t>
+          <t>Ministry of Defence</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Mizoram Gets Approval for New Road Works under PMGSY-IV to Strengthen Rural Connectivity</t>
+          <t>INAUGURAL BIMSTEC MARITIME SECURITY EXERCISE</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>pmgsy, pmgsy-iv, rural connectivity</t>
+          <t>maritime security</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 2 topics: pmgsy, pmgsy-iv, rural connectivity</t>
+          <t>Aligned with General Studies 3 topics: maritime security</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330725</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330850</t>
         </is>
       </c>
     </row>
@@ -904,32 +904,627 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Defence</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>AIR CHIEF MARSHAL ASHUTOSH DIXIT PVSM AVSM VM VSM ASSUMES CHARGE AS CHIEF OF THE AIR STAFF OF THE INDIAN AIR FORCE</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>indian air force</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 3 topics: indian air force</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330846</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Environment, Forest and Climate Change</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Union Ministry of Environment, Forest and Climate Change and its organisations successfully conclude Special Campaign 6</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>climate change</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 3 topics: climate change</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2331056</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Environment, Forest and Climate Change</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>High level CAQM Team reviews Paddy Straw Management Measures reviews in Sangrur, Patiala and Malerkotla of Punjab</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>climate change, caqm</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 3 topics: climate change, caqm</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2331055</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Environment, Forest and Climate Change</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Delhi Records Lowest Average AQI for October in the Last Eight Years at 166</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>climate change</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 3 topics: climate change</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2331032</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Finance</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>CBN Madhya Pradesh Unit conducts three major anti-drug operations; seizes 2,774.650 kg of poppy straw and five vehicles; arrests four persons</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Economic Governance &amp; Fiscal Policy</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>Strategic policy update from nodal ministry (Ministry of Finance): Economic Governance &amp; Fiscal Policy</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2331051</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>GS-1</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Health and Family Welfare</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Union Health Minister Shri J.P. Nadda administers Rashtriya Ekta Diwas pledge to commemorate the birth anniversary of Sardar Vallabhbhai Patel</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>birth anniversary, rashtriya ekta diwas, sardar vallabhbhai patel</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 1 topics: birth anniversary, rashtriya ekta diwas, sardar vallabhbhai patel</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330752</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>GS-1</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Home Affairs</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Union Home Minister and Minister of Cooperation Shri Amit Shah Flags off ‘Run for Unity’ in New Delhi on 'Rashtriya Ekta Diwas’on the occasion of 151st birth anniversary of Sardar Vallabhbhai Patel</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>birth anniversary, rashtriya ekta diwas, sardar vallabhbhai patel</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 1 topics: birth anniversary, rashtriya ekta diwas, sardar vallabhbhai patel</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330810</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Home Affairs</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>‘Kendriya Grihmantri Dakshata Padak’ awarded to 490 personnel of various States/UTs/CAPFs/CPOs for the year 2026</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>dakshata padak, kendriya grihmantri dakshata padak, capfs, cpos</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 3 topics: dakshata padak, kendriya grihmantri dakshata padak, capfs</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330728</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
           <t>GS-2</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Labour &amp; Employment</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>EPFO to Celebrate 74th Foundation Day in New Delhi Tomorrow</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>epfo</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 2 topics: epfo</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330894</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>GS-1</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Law and Justice</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Legislative Department Participates in ‘Run for Unity’ on Rashtriya Ekta Diwas.</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>rashtriya ekta diwas</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 1 topics: rashtriya ekta diwas</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330905</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>GS-2</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Panchayati Raj</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Union Minister Shri Rajiv Ranjan Singh Urges Concerted Efforts to Build ‘Atmanirbhar Panchayats’ at National Workshop on People’s Plan Campaign, in New Delhi</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>panchayati raj</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 2 topics: panchayati raj</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330751</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>GS-2</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Parliamentary Affairs</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Parliamentary Affairs Concludes Special Campaign 6.0 with Focus on Swachhata, Record Management and Digital Governance</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>governance</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 2 topics: governance</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330835</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>GS-2</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Personnel, Public Grievances &amp; Pensions</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Union Minister Dr. Jitendra Singh Positions IIPA’s Nationwide Outreach for Inclusive Capacity Building in Governance</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>governance</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 2 topics: governance</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330834</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>GS-2</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Rural Development</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Mizoram Gets Approval for New Road Works under PMGSY-IV to Strengthen Rural Connectivity</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>pmgsy, pmgsy-iv, rural connectivity</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 2 topics: pmgsy, pmgsy-iv, rural connectivity</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330725</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Textiles</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>Government of India extends Customs Duty Exemption on Cotton imports up to 31st December 2026</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>customs duty</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 3 topics: customs duty</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330823</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>GS-2</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>PIB Backgrounder</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D27" s="4" t="inlineStr">
         <is>
           <t>India’s Social Security Coverage</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E27" s="4" t="inlineStr">
         <is>
           <t>PIB Backgrounder, social security</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F27" s="4" t="inlineStr">
         <is>
           <t>PIB Backgrounder: Aligned with General Studies 2 topics: social security</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="G27" s="5" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330727</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Competition Commission of India</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>CCI approves acquisition of the equity share capital of IntelliSmart Infrastructure (Target) by Adani Energy Solutions Ltd. (Acquirer)</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>infrastructure</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 3 topics: infrastructure</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330819</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>GS-1</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Chemicals and Fertilizers - Department of Pharmaceuticals</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>Department of Pharmaceuticals Organises Plog Run under Fit India Freedom Run 7.0 on Rashtriya Ekta Diwas; Reaffirms Commitment to National Unity, Fitness, and Cleanliness</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>rashtriya ekta diwas</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 1 topics: rashtriya ekta diwas</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2331042</t>
         </is>
       </c>
     </row>
@@ -946,6 +1541,23 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId28"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -957,7 +1569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1006,12 +1618,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Relevant (UPSC)</t>
+          <t>Routine Fluff</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>GS-1</t>
+          <t>General/Administrative</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1021,12 +1633,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>PRESIDENT OF INDIA PAYS FLORAL TRIBUTES TO SARDAR VALLABHBHAI PATEL ON HIS BIRTH ANNIVERSARY</t>
+          <t>PRESIDENT OF INDIA GRACES the Dhwaj Stambh Pujan, Dhawaja Pujan and Dhwajarohan ceremony of Simhastha Maha Kumbh at Nashik</t>
         </is>
       </c>
       <c r="F2" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330757</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2331006</t>
         </is>
       </c>
     </row>
@@ -1041,22 +1653,22 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>GS-2</t>
+          <t>GS-1</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Lok Sabha Secretariat</t>
+          <t>President's Secretariat</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>LOK SABHA SPEAKER HAILS GAYATRI PARIVAR’S CONTRIBUTIONS TO INDIA'S SPIRITUAL RENAISSANCE, SOCIAL TRANSFORMATION AND NATION-BUILDING</t>
+          <t>PRESIDENT OF INDIA PAYS FLORAL TRIBUTES TO SARDAR VALLABHBHAI PATEL ON HIS BIRTH ANNIVERSARY</t>
         </is>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330789</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330757</t>
         </is>
       </c>
     </row>
@@ -1076,17 +1688,17 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Prime Minister's Office</t>
+          <t>Vice President's Secretariat</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Prime Minister pays tribute to Sardar Vallabhbhai Patel on his birth anniversary</t>
+          <t>Vice-President Shri C. P. Radhakrishnan attends ‘Sardar Katha’ at Uprashtrapati Bhavan; pays tribute to Sardar Vallabhbhai Patel on Rashtriya Ekta Diwas</t>
         </is>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330739</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330939</t>
         </is>
       </c>
     </row>
@@ -1096,27 +1708,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Relevant (UPSC)</t>
+          <t>Routine Fluff</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>GS-3</t>
+          <t>General/Administrative</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Prime Minister's Office</t>
+          <t>Vice President's Secretariat</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>PM congratulates ISRO scientists and engineers on successful launch of GSLV-F18 carrying NVS-03</t>
+          <t>Vice-President Shri C. P. Radhakrishnan Addresses 72nd Annual General Body Meeting of IIPA; Calls for Transformative Reforms in Public Administration to Realise Viksit Bharat @ 2047</t>
         </is>
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330735</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330891</t>
         </is>
       </c>
     </row>
@@ -1136,17 +1748,17 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>AYUSH</t>
+          <t>Prime Minister's Office</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Ministry of Ayush Promotes ‘Yoga for Unity’ on National Unity Day 2026</t>
+          <t>English rendering of PM’s speech at the Rashtriya Ekta Diwas programme in Kevadia, Gujarat</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330770</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2331035</t>
         </is>
       </c>
     </row>
@@ -1161,23 +1773,22 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>GS-3</t>
+          <t>GS-1</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Ministry of Agriculture &amp;
-Farmers Welfare</t>
+          <t>Prime Minister's Office</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>DARE–ICAR Intensifies Special Campaign 6.0, Promotes Cleanliness, Sustainable Waste Management and Better Office Spaces Across Institutes</t>
+          <t>Prime Minister Shri Narendra Modi participates in Rashtriya Ekta Diwas Celebrations marking the 151st birth anniversary of Sardar Vallabhbhai Patel</t>
         </is>
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330771</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2331033</t>
         </is>
       </c>
     </row>
@@ -1197,17 +1808,17 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Ministry of Health and Family Welfare</t>
+          <t>Prime Minister's Office</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Union Health Minister Shri J.P. Nadda administers Rashtriya Ekta Diwas pledge to commemorate the birth anniversary of Sardar Vallabhbhai Patel</t>
+          <t>Prime Minister pays tribute to Sardar Vallabhbhai Patel on his birth anniversary</t>
         </is>
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330752</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330739</t>
         </is>
       </c>
     </row>
@@ -1227,17 +1838,17 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Ministry of Home Affairs</t>
+          <t>Prime Minister's Office</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>‘Kendriya Grihmantri Dakshata Padak’ awarded to 490 personnel of various States/UTs/CAPFs/CPOs for the year 2026</t>
+          <t>PM congratulates ISRO scientists and engineers on successful launch of GSLV-F18 carrying NVS-03</t>
         </is>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330728</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330735</t>
         </is>
       </c>
     </row>
@@ -1247,27 +1858,27 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Relevant (UPSC)</t>
+          <t>Routine Fluff</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>GS-2</t>
+          <t>Routine/Ceremonial</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Ministry of Panchayati Raj</t>
+          <t>Lok Sabha Secretariat</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Union Minister Shri Rajiv Ranjan Singh Urges Concerted Efforts to Build ‘Atmanirbhar Panchayats’ at National Workshop on People’s Plan Campaign, in New Delhi</t>
+          <t>LOK SABHA SPEAKER CALLS UPON YOUTH TO UPHOLD NATIONAL UNITY AND INTEGRITY AND CONTRIBUTE TO BUILDING A DEVELOPED INDIA</t>
         </is>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330751</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2331012</t>
         </is>
       </c>
     </row>
@@ -1287,17 +1898,17 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Ministry of Rural Development</t>
+          <t>Lok Sabha Secretariat</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Mizoram Gets Approval for New Road Works under PMGSY-IV to Strengthen Rural Connectivity</t>
+          <t>LOK SABHA SPEAKER HAILS GAYATRI PARIVAR’S CONTRIBUTIONS TO INDIA'S SPIRITUAL RENAISSANCE, SOCIAL TRANSFORMATION AND NATION-BUILDING</t>
         </is>
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330725</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330789</t>
         </is>
       </c>
     </row>
@@ -1307,27 +1918,27 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Routine Fluff</t>
+          <t>Relevant (UPSC)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>General/Administrative</t>
+          <t>GS-1</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Ministry of Textiles</t>
+          <t>AYUSH</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Prime Minister visits CCIC Pavilion at Bharat Parv 2026 in Ekta Nagar, Gujarat</t>
+          <t>Ministry of Ayush Promotes ‘Yoga for Unity’ on National Unity Day 2026</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330737</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330770</t>
         </is>
       </c>
     </row>
@@ -1342,22 +1953,1103 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Ministry of Agriculture &amp;
+Farmers Welfare</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>DARE–ICAR Intensifies Special Campaign 6.0, Promotes Cleanliness, Sustainable Waste Management and Better Office Spaces Across Institutes</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330771</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Ministry of Corporate Affairs</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>MCA successfully concludes nationwide Special Campaign 6.0 on Swachchta</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330813</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Ministry of Defence</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>INAUGURAL BIMSTEC MARITIME SECURITY EXERCISE</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330850</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Ministry of Defence</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>AIR CHIEF MARSHAL AP SINGH SUPERANNUATES AFTER  42 YEARS OF DISTINGUISHED SERVICE TO THE NATION</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330848</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Ministry of Defence</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>AIR CHIEF MARSHAL ASHUTOSH DIXIT PVSM AVSM VM VSM ASSUMES CHARGE AS CHIEF OF THE AIR STAFF OF THE INDIAN AIR FORCE</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330846</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Ministry of Education</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>National CSR Meet for School Education organised through Vidyanjali</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330979</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Ministry of Education</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Last date for submission of applications under the National Means-cum-Merit Scholarship Scheme for academic year 2026-27 extended till November 15, 2026</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330936</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Ministry of Environment, Forest and Climate Change</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Union Ministry of Environment, Forest and Climate Change and its organisations successfully conclude Special Campaign 6</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2331056</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Ministry of Environment, Forest and Climate Change</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>High level CAQM Team reviews Paddy Straw Management Measures reviews in Sangrur, Patiala and Malerkotla of Punjab</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2331055</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Ministry of Environment, Forest and Climate Change</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Delhi Records Lowest Average AQI for October in the Last Eight Years at 166</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2331032</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Ministry of Finance</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Union Government releases tax devolution of ₹1,09,019 crore to State Governments, as one advance instalment of tax devolution in view of upcoming festive season and to enable States to accelerate capital spending and finance their development/ welfare related expenditure</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330997</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Ministry of Finance</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>CBN Madhya Pradesh Unit conducts three major anti-drug operations; seizes 2,774.650 kg of poppy straw and five vehicles; arrests four persons</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2331051</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>GS-1</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Ministry of Health and Family Welfare</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Union Health Minister Shri J.P. Nadda administers Rashtriya Ekta Diwas pledge to commemorate the birth anniversary of Sardar Vallabhbhai Patel</t>
+        </is>
+      </c>
+      <c r="F25" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330752</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>GS-1</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Ministry of Home Affairs</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Union Home Minister and Minister of Cooperation Shri Amit Shah Flags off ‘Run for Unity’ in New Delhi on 'Rashtriya Ekta Diwas’on the occasion of 151st birth anniversary of Sardar Vallabhbhai Patel</t>
+        </is>
+      </c>
+      <c r="F26" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330810</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Ministry of Home Affairs</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>‘Kendriya Grihmantri Dakshata Padak’ awarded to 490 personnel of various States/UTs/CAPFs/CPOs for the year 2026</t>
+        </is>
+      </c>
+      <c r="F27" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330728</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Ministry of Housing &amp; Urban Affairs</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>MoHUA Conducts Participatory Workshop to Chart a Shared Roadmap for Clean Delhi</t>
+        </is>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330869</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
           <t>GS-2</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Ministry of Labour &amp; Employment</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>EPFO to Celebrate 74th Foundation Day in New Delhi Tomorrow</t>
+        </is>
+      </c>
+      <c r="F29" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330894</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>GS-1</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Ministry of Law and Justice</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Legislative Department Participates in ‘Run for Unity’ on Rashtriya Ekta Diwas.</t>
+        </is>
+      </c>
+      <c r="F30" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330905</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>GS-2</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Ministry of Panchayati Raj</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Union Minister Shri Rajiv Ranjan Singh Urges Concerted Efforts to Build ‘Atmanirbhar Panchayats’ at National Workshop on People’s Plan Campaign, in New Delhi</t>
+        </is>
+      </c>
+      <c r="F31" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330751</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>GS-2</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Ministry of Parliamentary Affairs</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Ministry of Parliamentary Affairs Concludes Special Campaign 6.0 with Focus on Swachhata, Record Management and Digital Governance</t>
+        </is>
+      </c>
+      <c r="F32" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330835</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>GS-2</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Ministry of Personnel, Public Grievances &amp; Pensions</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Union Minister Dr. Jitendra Singh Positions IIPA’s Nationwide Outreach for Inclusive Capacity Building in Governance</t>
+        </is>
+      </c>
+      <c r="F33" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330834</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Ministry of Rural Development</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>“Every drop of rain must be conserved to make villages water-secure and self-reliant”- Secretary, DoLR, Shri Dilip Kumar</t>
+        </is>
+      </c>
+      <c r="F34" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330839</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>GS-2</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Ministry of Rural Development</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Mizoram Gets Approval for New Road Works under PMGSY-IV to Strengthen Rural Connectivity</t>
+        </is>
+      </c>
+      <c r="F35" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330725</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Ministry of Ports, Shipping and Waterways</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Sarbananda Sonowal Administers National Unity Pledge to Ministry Officials, Student Cadets</t>
+        </is>
+      </c>
+      <c r="F36" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330978</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Ministry of Social Justice &amp; Empowerment</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Ministry Of Social Justice And Empowerment Issues Factual Report With Regard To The Claim—Appearing In A Report Published In The Central Chronicle (Bhopal) On October 31, 2026</t>
+        </is>
+      </c>
+      <c r="F37" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2331004</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Ministry of Social Justice &amp; Empowerment</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>15 Day Shilp Samagam Mela 2026 To Start At Dilli Haat, New Delhi, From Tomorrow</t>
+        </is>
+      </c>
+      <c r="F38" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330929</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Ministry of Textiles</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Government of India extends Customs Duty Exemption on Cotton imports up to 31st December 2026</t>
+        </is>
+      </c>
+      <c r="F39" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330823</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Ministry of Textiles</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Prime Minister visits CCIC Pavilion at Bharat Parv 2026 in Ekta Nagar, Gujarat</t>
+        </is>
+      </c>
+      <c r="F40" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330737</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Ministry of Youth Affairs and Sports</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>MY Bharat - NSS Mobilises Over 96,700 Youth  in Nationwide Cyclothons and Walkathons under Nasha Mukt Yuva Abhiyan</t>
+        </is>
+      </c>
+      <c r="F41" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2331041</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Ministry of Youth Affairs and Sports</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>MY Bharat’s ‘Viksit Bharat Yuva Samvad: Know Your Vote’ Campaign Engages Over 11,000 Youth Through 62 Programmes Across 16 States/UTs</t>
+        </is>
+      </c>
+      <c r="F42" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330991</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>GS-2</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
         <is>
           <t>PIB Backgrounder</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E43" t="inlineStr">
         <is>
           <t>India’s Social Security Coverage</t>
         </is>
       </c>
-      <c r="F13" s="9" t="inlineStr">
+      <c r="F43" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330727</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Competition Commission of India</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>CCI approves acquisition of certain shareholding in Navi Ltd by MIH Payments Holdings B.V.</t>
+        </is>
+      </c>
+      <c r="F44" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330818</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Competition Commission of India</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>CCI approves acquisition of the equity share capital of IntelliSmart Infrastructure (Target) by Adani Energy Solutions Ltd. (Acquirer)</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330819</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Competition Commission of India</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>CCI approves merger of Sapphire Foods India with and into Devyani International and related transactions</t>
+        </is>
+      </c>
+      <c r="F46" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330817</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Competition Commission of India</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>CCI approves acquisition of 100% of the issued share capital of Solenergi Power (Target) by Aditya Birla Renewables Ltd (Acquirer)</t>
+        </is>
+      </c>
+      <c r="F47" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330816</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Competition Commission of India</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>CCI approves acquisition of certain stake in Vodafone Group PLC by Vega SAS</t>
+        </is>
+      </c>
+      <c r="F48" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2330815</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>GS-1</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Ministry of Chemicals and Fertilizers - Department of Pharmaceuticals</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Department of Pharmaceuticals Organises Plog Run under Fit India Freedom Run 7.0 on Rashtriya Ekta Diwas; Reaffirms Commitment to National Unity, Fitness, and Cleanliness</t>
+        </is>
+      </c>
+      <c r="F49" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2331042</t>
         </is>
       </c>
     </row>
@@ -1375,6 +3067,42 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F49" r:id="rId48"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>